<commit_message>
chore(scripts): make demo sheets look like a real class
With the status bands in place, the old sample numbers put 85% of the
demo class at risk, which does not look like a real class in front of
faculty. Most students now do well. About one in five is short on
attendance in one subject, and a few fail or miss a Mid-Sem, so every
tile and badge still has something to show.
</commit_message>
<xml_diff>
--- a/samples/ce-a-sem-6.xlsx
+++ b/samples/ce-a-sem-6.xlsx
@@ -496,22 +496,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Theory=72,Practical=76,Marks=4</t>
+          <t>Theory=84,Practical=86,Marks=7</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Theory=83,Practical=79,Marks=9</t>
+          <t>Theory=95,Practical=89,Marks=12</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Theory=94,Marks=14</t>
+          <t>Theory=84,Marks=17</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Theory=71,Practical=85,Marks=19</t>
+          <t>Theory=95,Practical=95,Marks=8</t>
         </is>
       </c>
     </row>
@@ -541,22 +541,22 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Theory=79,Practical=81,Marks=7</t>
+          <t>Theory=91,Practical=91,Marks=10</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Theory=90,Practical=84,Marks=12</t>
+          <t>Theory=80,Practical=94,Marks=15</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Theory=67,Marks=17</t>
+          <t>Theory=91,Marks=20</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Theory=78,Practical=90,Marks=5</t>
+          <t>Theory=80,Practical=80,Marks=11</t>
         </is>
       </c>
     </row>
@@ -586,22 +586,22 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Theory=86,Practical=86,Marks=10</t>
+          <t>Theory=98,Practical=96,Marks=13</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Theory=97,Practical=89,Marks=15</t>
+          <t>Theory=87,Practical=99,Marks=18</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Theory=74,Marks=20</t>
+          <t>Theory=98,Marks=9</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Theory=85,Practical=95,Marks=AB</t>
+          <t>Theory=87,Practical=85,Marks=AB</t>
         </is>
       </c>
     </row>
@@ -631,22 +631,22 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Theory=93,Practical=91,Marks=13</t>
+          <t>Theory=83,Practical=81,Marks=16</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Theory=70,Practical=94,Marks=18</t>
+          <t>Theory=94,Practical=84,Marks=7</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Theory=81,Marks=6</t>
+          <t>Theory=83,Marks=12</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Theory=92,Practical=70,Marks=11</t>
+          <t>Theory=94,Practical=90,Marks=17</t>
         </is>
       </c>
     </row>
@@ -676,22 +676,22 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Theory=66,Practical=96,Marks=16</t>
+          <t>Theory=68,Practical=86,Marks=19</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Theory=77,Practical=99,Marks=4</t>
+          <t>Theory=79,Practical=89,Marks=10</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Theory=88,Marks=9</t>
+          <t>Theory=90,Marks=15</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Theory=99,Practical=75,Marks=14</t>
+          <t>Theory=79,Practical=95,Marks=3</t>
         </is>
       </c>
     </row>
@@ -721,22 +721,22 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Theory=73,Practical=71,Marks=19</t>
+          <t>Theory=97,Practical=91,Marks=8</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Theory=84,Practical=74,Marks=7</t>
+          <t>Theory=86,Practical=94,Marks=13</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Theory=95,Marks=AB</t>
+          <t>Theory=97,Marks=AB</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Theory=72,Practical=80,Marks=17</t>
+          <t>Theory=86,Practical=80,Marks=9</t>
         </is>
       </c>
     </row>
@@ -766,22 +766,22 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Theory=80,Practical=76,Marks=5</t>
+          <t>Theory=82,Practical=96,Marks=11</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Theory=91,Practical=79,Marks=10</t>
+          <t>Theory=93,Practical=99,Marks=5</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Theory=68,Marks=15</t>
+          <t>Theory=82,Marks=7</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Theory=79,Practical=85,Marks=20</t>
+          <t>Theory=93,Practical=85,Marks=12</t>
         </is>
       </c>
     </row>
@@ -811,22 +811,22 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Theory=87,Practical=81,Marks=8</t>
+          <t>Theory=89,Practical=81,Marks=6</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Theory=98,Practical=84,Marks=13</t>
+          <t>Theory=78,Practical=84,Marks=19</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Theory=75,Marks=18</t>
+          <t>Theory=89,Marks=10</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Theory=86,Practical=90,Marks=6</t>
+          <t>Theory=78,Practical=90,Marks=15</t>
         </is>
       </c>
     </row>
@@ -856,22 +856,22 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Theory=94,Practical=86,Marks=11</t>
+          <t>Theory=96,Practical=86,Marks=17</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Theory=71,Practical=89,Marks=AB</t>
+          <t>Theory=85,Practical=89,Marks=AB</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Theory=82,Marks=4</t>
+          <t>Theory=96,Marks=13</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Theory=93,Practical=95,Marks=9</t>
+          <t>Theory=85,Practical=95,Marks=18</t>
         </is>
       </c>
     </row>
@@ -901,22 +901,22 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Theory=67,Practical=91,Marks=14</t>
+          <t>Theory=65,Practical=91,Marks=20</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Theory=78,Practical=94,Marks=19</t>
+          <t>Theory=92,Practical=94,Marks=11</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Theory=89,Marks=7</t>
+          <t>Theory=81,Marks=16</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Theory=66,Practical=70,Marks=12</t>
+          <t>Theory=92,Practical=80,Marks=7</t>
         </is>
       </c>
     </row>
@@ -946,22 +946,22 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Theory=74,Practical=96,Marks=17</t>
+          <t>Theory=88,Practical=96,Marks=9</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Theory=85,Practical=99,Marks=5</t>
+          <t>Theory=99,Practical=99,Marks=14</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Theory=96,Marks=10</t>
+          <t>Theory=88,Marks=19</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Theory=73,Practical=75,Marks=15</t>
+          <t>Theory=99,Practical=85,Marks=10</t>
         </is>
       </c>
     </row>
@@ -991,22 +991,22 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Theory=81,Practical=71,Marks=AB</t>
+          <t>Theory=95,Practical=81,Marks=AB</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Theory=92,Practical=74,Marks=8</t>
+          <t>Theory=84,Practical=84,Marks=17</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Theory=69,Marks=13</t>
+          <t>Theory=95,Marks=8</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Theory=80,Practical=80,Marks=18</t>
+          <t>Theory=84,Practical=90,Marks=13</t>
         </is>
       </c>
     </row>
@@ -1036,22 +1036,22 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Theory=88,Practical=76,Marks=6</t>
+          <t>Theory=80,Practical=86,Marks=15</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Theory=99,Practical=79,Marks=11</t>
+          <t>Theory=91,Practical=89,Marks=20</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Theory=76,Marks=16</t>
+          <t>Theory=80,Marks=11</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Theory=87,Practical=85,Marks=4</t>
+          <t>Theory=91,Practical=95,Marks=16</t>
         </is>
       </c>
     </row>
@@ -1081,22 +1081,22 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Theory=95,Practical=81,Marks=9</t>
+          <t>Theory=87,Practical=91,Marks=18</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Theory=72,Practical=84,Marks=14</t>
+          <t>Theory=98,Practical=94,Marks=9</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Theory=83,Marks=19</t>
+          <t>Theory=87,Marks=14</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Theory=94,Practical=90,Marks=7</t>
+          <t>Theory=98,Practical=80,Marks=19</t>
         </is>
       </c>
     </row>
@@ -1126,22 +1126,22 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Theory=68,Practical=86,Marks=12</t>
+          <t>Theory=70,Practical=96,Marks=7</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Theory=79,Practical=89,Marks=17</t>
+          <t>Theory=83,Practical=99,Marks=12</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Theory=90,Marks=5</t>
+          <t>Theory=94,Marks=17</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Theory=67,Practical=95,Marks=10</t>
+          <t>Theory=83,Practical=85,Marks=8</t>
         </is>
       </c>
     </row>
@@ -1171,22 +1171,22 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Theory=75,Practical=91,Marks=15</t>
+          <t>Theory=79,Practical=81,Marks=10</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Theory=86,Practical=94,Marks=20</t>
+          <t>Theory=90,Practical=84,Marks=15</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Theory=97,Marks=8</t>
+          <t>Theory=79,Marks=20</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Theory=74,Practical=70,Marks=13</t>
+          <t>Theory=90,Practical=90,Marks=11</t>
         </is>
       </c>
     </row>
@@ -1216,22 +1216,22 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Theory=82,Practical=96,Marks=18</t>
+          <t>Theory=86,Practical=86,Marks=13</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Theory=93,Practical=99,Marks=6</t>
+          <t>Theory=97,Practical=89,Marks=18</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Theory=70,Marks=11</t>
+          <t>Theory=86,Marks=9</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Theory=81,Practical=75,Marks=16</t>
+          <t>Theory=97,Practical=95,Marks=14</t>
         </is>
       </c>
     </row>
@@ -1261,22 +1261,22 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Theory=89,Practical=71,Marks=4</t>
+          <t>Theory=93,Practical=91,Marks=16</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Theory=66,Practical=74,Marks=9</t>
+          <t>Theory=82,Practical=94,Marks=7</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Theory=77,Marks=14</t>
+          <t>Theory=93,Marks=12</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Theory=88,Practical=80,Marks=19</t>
+          <t>Theory=82,Practical=80,Marks=4</t>
         </is>
       </c>
     </row>
@@ -1306,22 +1306,22 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Theory=96,Practical=76,Marks=7</t>
+          <t>Theory=78,Practical=96,Marks=19</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Theory=73,Practical=79,Marks=12</t>
+          <t>Theory=89,Practical=99,Marks=10</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Theory=84,Marks=17</t>
+          <t>Theory=78,Marks=5</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Theory=95,Practical=85,Marks=5</t>
+          <t>Theory=89,Practical=85,Marks=20</t>
         </is>
       </c>
     </row>
@@ -1351,22 +1351,22 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Theory=69,Practical=81,Marks=10</t>
+          <t>Theory=67,Practical=81,Marks=8</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Theory=80,Practical=84,Marks=15</t>
+          <t>Theory=96,Practical=84,Marks=6</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Theory=91,Marks=20</t>
+          <t>Theory=85,Marks=18</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Theory=68,Practical=90,Marks=AB</t>
+          <t>Theory=96,Practical=90,Marks=AB</t>
         </is>
       </c>
     </row>

</xml_diff>